<commit_message>
Update Excel statements to format PNG trade graph links as native =HYPERLINK formula
</commit_message>
<xml_diff>
--- a/Reports/Intraday_Strategy_Account_Statement.xlsx
+++ b/Reports/Intraday_Strategy_Account_Statement.xlsx
@@ -646,10 +646,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O3" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0001_ADANIENT.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -707,10 +706,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O4" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0002_ADANIENT.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -768,10 +766,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O5" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0003_APOLLOHOSP.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -829,10 +826,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O6" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0004_AUROPHARMA.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -890,10 +886,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O7" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0005_BAJFINANCE.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -951,10 +946,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O8" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0006_BAJFINANCE.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -1012,10 +1006,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O9" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O9" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0007_BALKRISIND.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -1073,10 +1066,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O10" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0008_BANDHANBNK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -1134,10 +1126,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O11" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O11" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0009_BEL.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -1195,10 +1186,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O12" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0010_BEL.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -1256,10 +1246,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O13" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O13" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0011_BEL.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1317,10 +1306,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O14" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0012_BEL.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -1378,10 +1366,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O15" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O15" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0013_BEL.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -1439,10 +1426,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O16" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O16" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0014_BEL.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -1500,10 +1486,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O17" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O17" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0015_BEML.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -1561,10 +1546,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O18" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O18" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0016_BHARATFORG.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1622,10 +1606,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O19" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O19" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0017_BHARATFORG.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1683,10 +1666,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O20" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O20" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0018_BHARATFORG.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1744,10 +1726,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O21" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O21" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0019_BHARTIARTL.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1805,10 +1786,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O22" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O22" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0020_BHARTIARTL.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -1866,10 +1846,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O23" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O23" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0021_BHEL.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -1927,10 +1906,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O24" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O24" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0022_BPCL.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1988,10 +1966,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O25" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O25" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0023_BPCL.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -2049,10 +2026,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O26" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O26" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0024_COALINDIA.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -2110,10 +2086,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O27" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O27" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0025_DIVISLAB.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -2171,10 +2146,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O28" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O28" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0026_DIXON.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -2232,10 +2206,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O29" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O29" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0027_DRREDDY.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -2293,10 +2266,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O30" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O30" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0028_DRREDDY.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -2354,10 +2326,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O31" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O31" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0029_EICHERMOT.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -2415,10 +2386,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O32" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O32" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0030_EICHERMOT.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -2476,10 +2446,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O33" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O33" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0031_EICHERMOT.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -2537,10 +2506,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O34" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O34" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0032_EICHERMOT.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -2598,10 +2566,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O35" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O35" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0033_GAIL.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -2659,10 +2626,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O36" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O36" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0034_GAIL.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -2720,10 +2686,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O37" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O37" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0035_HCLTECH.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -2781,10 +2746,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O38" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O38" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0036_HCLTECH.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -2842,10 +2806,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O39" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O39" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0037_HDFCBANK.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -2903,10 +2866,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O40" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O40" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0038_HDFCBANK.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -2964,10 +2926,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O41" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O41" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0039_HEXT.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -3025,10 +2986,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O42" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O42" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0040_HINDUNILVR.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -3086,10 +3046,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O43" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O43" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0041_HINDUNILVR.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -3147,10 +3106,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O44" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O44" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0042_HONASA.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -3208,10 +3166,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O45" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O45" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0043_HONASA.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -3269,10 +3226,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O46" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O46" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0044_HONASA.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -3330,10 +3286,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O47" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O47" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0045_HONASA.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -3391,10 +3346,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O48" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O48" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0046_ICICIBANK.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -3452,10 +3406,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O49" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O49" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0047_ICICIBANK.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -3513,10 +3466,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O50" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O50" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0048_IDEA.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="51">
@@ -3574,10 +3526,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O51" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O51" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0049_INFY.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -3635,10 +3586,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O52" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O52" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0050_INFY.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="53">
@@ -3696,10 +3646,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O53" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O53" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0051_ITC.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="54">
@@ -3757,10 +3706,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O54" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O54" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0052_JSWENERGY.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="55">
@@ -3818,10 +3766,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O55" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O55" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0053_JSWENERGY.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="56">
@@ -3879,10 +3826,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O56" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O56" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0054_KOTAKBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="57">
@@ -3940,10 +3886,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O57" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O57" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0055_KOTAKBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="58">
@@ -4001,10 +3946,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O58" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O58" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0056_KOTAKBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -4062,10 +4006,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O59" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O59" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0057_KOTAKBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="60">
@@ -4123,10 +4066,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O60" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O60" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0058_KOTAKBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="61">
@@ -4184,10 +4126,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O61" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O61" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0059_KOTAKBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="62">
@@ -4245,10 +4186,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O62" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O62" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0060_KOTAKBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="63">
@@ -4306,10 +4246,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O63" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O63" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0061_KTKBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -4367,10 +4306,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O64" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O64" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0062_KTKBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="65">
@@ -4428,10 +4366,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O65" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O65" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0063_LUPIN.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="66">
@@ -4489,10 +4426,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O66" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O66" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0064_LUPIN.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -4550,10 +4486,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O67" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O67" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0065_LUPIN.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="68">
@@ -4611,10 +4546,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O68" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O68" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0066_LUPIN.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="69">
@@ -4672,10 +4606,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O69" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O69" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0067_LUPIN.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="70">
@@ -4733,10 +4666,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O70" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O70" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0068_LUPIN.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="71">
@@ -4794,10 +4726,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O71" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O71" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0069_LUPIN.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="72">
@@ -4855,10 +4786,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O72" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O72" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0070_LUPIN.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="73">
@@ -4916,10 +4846,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O73" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O73" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0071_MAXHEALTH.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="74">
@@ -4977,10 +4906,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O74" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O74" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0072_NYKAA.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="75">
@@ -5038,10 +4966,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O75" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O75" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0073_NYKAA.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="76">
@@ -5099,10 +5026,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O76" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O76" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0074_NYKAA.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="77">
@@ -5160,10 +5086,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O77" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O77" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0075_RELIANCE.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="78">
@@ -5221,10 +5146,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O78" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O78" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0076_RELIANCE.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="79">
@@ -5282,10 +5206,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O79" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O79" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0077_RELIANCE.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="80">
@@ -5343,10 +5266,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O80" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O80" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0078_RELIANCE.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="81">
@@ -5404,10 +5326,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O81" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O81" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0079_RELIANCE.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="82">
@@ -5465,10 +5386,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O82" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O82" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0080_RELIANCE.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="83">
@@ -5526,10 +5446,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O83" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O83" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0081_RELIANCE.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="84">
@@ -5587,10 +5506,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O84" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O84" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0082_RELIANCE.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="85">
@@ -5648,10 +5566,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O85" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O85" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0083_RVNL.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="86">
@@ -5709,10 +5626,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O86" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O86" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0084_SIEMENS.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="87">
@@ -5770,10 +5686,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O87" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O87" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0085_SIEMENS.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="88">
@@ -5831,10 +5746,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O88" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O88" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0086_SIEMENS.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="89">
@@ -5892,10 +5806,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O89" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O89" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0087_SJVN.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="90">
@@ -5953,10 +5866,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O90" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O90" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0088_SJVN.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="91">
@@ -6014,10 +5926,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O91" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O91" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0089_SUNPHARMA.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="92">
@@ -6075,10 +5986,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O92" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O92" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0090_SUNPHARMA.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="93">
@@ -6136,10 +6046,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O93" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O93" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0091_TATACOMM.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="94">
@@ -6197,10 +6106,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O94" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O94" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0092_TATACOMM.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="95">
@@ -6258,10 +6166,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O95" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O95" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0093_TATAPOWER.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="96">
@@ -6319,10 +6226,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O96" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O96" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0094_TATAPOWER.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="97">
@@ -6380,10 +6286,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O97" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O97" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0095_TATAPOWER.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="98">
@@ -6441,10 +6346,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O98" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O98" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0096_TECHM.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="99">
@@ -6502,10 +6406,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O99" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O99" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0097_TECHM.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="100">
@@ -6563,10 +6466,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O100" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O100" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0098_TECHM.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="101">
@@ -6624,10 +6526,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O101" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O101" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0099_TMCV.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="102">
@@ -6685,10 +6586,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O102" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O102" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0100_TORNTPOWER.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="103">
@@ -6746,10 +6646,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O103" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O103" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0101_TORNTPOWER.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="104">
@@ -6807,10 +6706,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O104" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O104" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0102_TRENT.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="105">
@@ -6868,10 +6766,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O105" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O105" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0103_TRENT.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="106">
@@ -6929,10 +6826,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O106" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O106" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0104_TRENT.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="107">
@@ -6990,10 +6886,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O107" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O107" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0105_TRENT.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="108">
@@ -7051,10 +6946,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O108" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O108" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0106_VOLTAS.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="109">
@@ -7112,10 +7006,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O109" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O109" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0107_VOLTAS.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="110">
@@ -7173,10 +7066,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O110" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O110" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0108_VOLTAS.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="111">
@@ -7234,10 +7126,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O111" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O111" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0109_VOLTAS.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="112">
@@ -7295,10 +7186,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O112" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O112" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0110_VOLTAS.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="113">
@@ -7356,10 +7246,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O113" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O113" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0111_WIPRO.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="114">
@@ -7417,10 +7306,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O114" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O114" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0112_YESBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="115">
@@ -7478,10 +7366,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O115" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O115" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0113_YESBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="116">
@@ -7539,10 +7426,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O116" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O116" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0114_YESBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="117">
@@ -7600,10 +7486,9 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="O117" s="4" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O117" s="4">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0115_YESBANK.NS_LOSS.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
     <row r="118">
@@ -7661,10 +7546,9 @@
           <t>PROFIT</t>
         </is>
       </c>
-      <c r="O118" s="5" t="inlineStr">
-        <is>
-          <t>View Intraday Plot Chart</t>
-        </is>
+      <c r="O118" s="5">
+        <f>HYPERLINK("file:///C:/DATA/CODE/Stocks/BackTest/Plots/intraday_trades/Intraday_Trade_0116_ZYDUSLIFE.NS_PROFIT.png", "View Intraday Plot Chart")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>